<commit_message>
Second part is comlited
</commit_message>
<xml_diff>
--- a/Check.xlsx
+++ b/Check.xlsx
@@ -611,7 +611,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -661,6 +661,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -946,7 +950,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="24.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="8"/>
       <c r="B3" s="9" t="s">
         <v>8</v>
@@ -958,7 +962,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="24.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8"/>
       <c r="B4" s="9" t="s">
         <v>9</v>
@@ -1018,7 +1022,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="24.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="8"/>
       <c r="B9" s="9" t="s">
         <v>14</v>
@@ -1030,7 +1034,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="24.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="8"/>
       <c r="B10" s="9" t="s">
         <v>15</v>
@@ -1326,7 +1330,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="24.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="8"/>
       <c r="B34" s="9" t="s">
         <v>44</v>
@@ -1496,7 +1500,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="24.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="48" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="8"/>
       <c r="B48" s="9" t="s">
         <v>56</v>
@@ -1508,7 +1512,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="49" customFormat="false" ht="24.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="49" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="8"/>
       <c r="B49" s="9" t="s">
         <v>57</v>
@@ -1520,7 +1524,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="50" customFormat="false" ht="24.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="50" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="8"/>
       <c r="B50" s="9" t="s">
         <v>58</v>
@@ -1532,7 +1536,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="51" customFormat="false" ht="24.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="51" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="8"/>
       <c r="B51" s="9" t="s">
         <v>59</v>
@@ -1544,7 +1548,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="52" customFormat="false" ht="24.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="52" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="8"/>
       <c r="B52" s="9" t="s">
         <v>60</v>
@@ -1666,7 +1670,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="62" customFormat="false" ht="24.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="62" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="8"/>
       <c r="B62" s="9" t="s">
         <v>64</v>
@@ -1750,7 +1754,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="69" customFormat="false" ht="24.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="69" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="8"/>
       <c r="B69" s="9" t="s">
         <v>51</v>
@@ -2096,8 +2100,8 @@
       <c r="C97" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="D97" s="12" t="s">
-        <v>69</v>
+      <c r="D97" s="13" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>